<commit_message>
COD payment request: department head Nguyen Tuan Viet, drop department row
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/src/main/resources/templates/cod-payment-request.xlsx
+++ b/src/main/resources/templates/cod-payment-request.xlsx
@@ -1623,14 +1623,7 @@
       <c r="H8" s="43"/>
       <c r="I8" s="42"/>
     </row>
-    <row r="9" ht="30.75" customHeight="1" spans="2:9">
-      <c r="B9" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="C9" s="42"/>
-      <c r="H9" s="43"/>
-      <c r="I9" s="42"/>
-    </row>
+    <row r="9" ht="30.75" hidden="1" customHeight="1" spans="2:9"/>
     <row r="10" ht="30.75" customHeight="1" spans="2:9">
       <c r="B10" s="5" t="str">
         <f>"Lý do xin thanh toán: "&amp;C14</f>
@@ -1848,6 +1841,9 @@
       </c>
     </row>
     <row r="32" spans="2:9">
+      <c r="E32" s="34"/>
+      <c r="F32" s="34"/>
+      <c r="G32" s="34"/>
       <c r="I32" s="34"/>
     </row>
     <row r="33" spans="9:9">
@@ -1857,7 +1853,7 @@
       <c r="I34" s="34"/>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="H1:I1"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="B5:I5"/>
@@ -1866,6 +1862,7 @@
     <mergeCell ref="E27:G27"/>
     <mergeCell ref="C28:D28"/>
     <mergeCell ref="E28:G28"/>
+    <mergeCell ref="E32:G32"/>
   </mergeCells>
   <pageMargins left="0.36" right="0.12" top="0.27" bottom="0.29" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="61" orientation="portrait"/>

</xml_diff>